<commit_message>
Daily NSE scan: 2026-09-11
</commit_message>
<xml_diff>
--- a/output/2026-09-11/enriched_analysis.xlsx
+++ b/output/2026-09-11/enriched_analysis.xlsx
@@ -819,7 +819,7 @@
         <v>2655</v>
       </c>
       <c r="R2" t="n">
-        <v>9.130000000000001</v>
+        <v>9.15</v>
       </c>
       <c r="S2" t="n">
         <v>36</v>
@@ -995,13 +995,13 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.308</v>
+        <v>0.317</v>
       </c>
       <c r="Q3" t="n">
-        <v>922</v>
+        <v>897</v>
       </c>
       <c r="R3" t="n">
-        <v>26.4</v>
+        <v>25.7</v>
       </c>
       <c r="S3" t="n">
         <v>19</v>
@@ -1177,13 +1177,13 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>3.63</v>
+        <v>3.623</v>
       </c>
       <c r="Q4" t="n">
-        <v>2918</v>
+        <v>2923</v>
       </c>
       <c r="R4" t="n">
-        <v>22.8</v>
+        <v>22.9</v>
       </c>
       <c r="S4" t="n">
         <v>75</v>
@@ -1359,13 +1359,13 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0.062</v>
+        <v>0.064</v>
       </c>
       <c r="Q5" t="n">
-        <v>1323</v>
+        <v>1288</v>
       </c>
       <c r="R5" t="n">
-        <v>17.8</v>
+        <v>17.4</v>
       </c>
       <c r="S5" t="n">
         <v>55</v>
@@ -1541,13 +1541,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.727</v>
+        <v>0.72</v>
       </c>
       <c r="Q6" t="n">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="R6" t="n">
-        <v>8.9</v>
+        <v>8.94</v>
       </c>
       <c r="S6" t="n">
         <v>17</v>
@@ -1723,13 +1723,13 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>0.048</v>
+        <v>0.049</v>
       </c>
       <c r="Q7" t="n">
-        <v>16047</v>
+        <v>15834</v>
       </c>
       <c r="R7" t="n">
-        <v>20.3</v>
+        <v>20.1</v>
       </c>
       <c r="S7" t="n">
         <v>16</v>
@@ -1908,7 +1908,7 @@
         <v>0.145</v>
       </c>
       <c r="Q8" t="n">
-        <v>2165</v>
+        <v>2172</v>
       </c>
       <c r="R8" t="n">
         <v>19</v>
@@ -2090,7 +2090,7 @@
         <v>0.006</v>
       </c>
       <c r="Q9" t="n">
-        <v>4358</v>
+        <v>4257</v>
       </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
@@ -2267,13 +2267,13 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>0.31</v>
+        <v>0.317</v>
       </c>
       <c r="Q10" t="n">
-        <v>2735</v>
+        <v>2681</v>
       </c>
       <c r="R10" t="n">
-        <v>22.4</v>
+        <v>22</v>
       </c>
       <c r="S10" t="n">
         <v>8</v>
@@ -2449,13 +2449,13 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>0.046</v>
+        <v>0.045</v>
       </c>
       <c r="Q11" t="n">
-        <v>15794</v>
+        <v>15960</v>
       </c>
       <c r="R11" t="n">
-        <v>40.2</v>
+        <v>40.6</v>
       </c>
       <c r="S11" t="n">
         <v>83</v>
@@ -2631,13 +2631,13 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>0.077</v>
+        <v>0.08</v>
       </c>
       <c r="Q12" t="n">
-        <v>443</v>
+        <v>427</v>
       </c>
       <c r="R12" t="n">
-        <v>13.1</v>
+        <v>12.6</v>
       </c>
       <c r="S12" t="n">
         <v>-8</v>
@@ -2813,13 +2813,13 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0.549</v>
+        <v>0.57</v>
       </c>
       <c r="Q13" t="n">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="R13" t="n">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="S13" t="n">
         <v>22</v>
@@ -2995,13 +2995,13 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>0.259</v>
+        <v>0.263</v>
       </c>
       <c r="Q14" t="n">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="R14" t="n">
-        <v>27.1</v>
+        <v>26.6</v>
       </c>
       <c r="S14" t="n">
         <v>21</v>
@@ -3177,10 +3177,10 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>0.628</v>
+        <v>0.655</v>
       </c>
       <c r="Q15" t="n">
-        <v>339</v>
+        <v>325</v>
       </c>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="n">
@@ -3357,13 +3357,13 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.089</v>
       </c>
       <c r="Q16" t="n">
-        <v>304</v>
+        <v>293</v>
       </c>
       <c r="R16" t="n">
-        <v>32.5</v>
+        <v>31.4</v>
       </c>
       <c r="S16" t="n">
         <v>24</v>
@@ -3539,13 +3539,13 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>0.136</v>
+        <v>0.135</v>
       </c>
       <c r="Q17" t="n">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="R17" t="n">
-        <v>5.93</v>
+        <v>5.98</v>
       </c>
       <c r="S17" t="n">
         <v>118</v>
@@ -3717,13 +3717,13 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>0.179</v>
+        <v>0.177</v>
       </c>
       <c r="Q18" t="n">
-        <v>1680</v>
+        <v>1703</v>
       </c>
       <c r="R18" t="n">
-        <v>58.6</v>
+        <v>59.4</v>
       </c>
       <c r="S18" t="n">
         <v>7</v>
@@ -3902,10 +3902,10 @@
         <v>0.007</v>
       </c>
       <c r="Q19" t="n">
-        <v>5735</v>
+        <v>5648</v>
       </c>
       <c r="R19" t="n">
-        <v>9.69</v>
+        <v>9.57</v>
       </c>
       <c r="S19" t="n">
         <v>43</v>
@@ -4081,13 +4081,13 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>0.036</v>
+        <v>0.037</v>
       </c>
       <c r="Q20" t="n">
-        <v>3715</v>
+        <v>3587</v>
       </c>
       <c r="R20" t="n">
-        <v>22</v>
+        <v>21.3</v>
       </c>
       <c r="S20" t="n">
         <v>-4</v>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PNGS Reva Diamond Jewellery Limited</t>
+          <t>PNGS REVA DIAMOND JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -4266,7 +4266,7 @@
         <v>0.109</v>
       </c>
       <c r="Q21" t="n">
-        <v>1600</v>
+        <v>1601</v>
       </c>
       <c r="R21" t="n">
         <v>19</v>
@@ -4443,13 +4443,13 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>2.231</v>
+        <v>2.252</v>
       </c>
       <c r="Q22" t="n">
-        <v>2670</v>
+        <v>2646</v>
       </c>
       <c r="R22" t="n">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="S22" t="n">
         <v>6</v>
@@ -4605,33 +4605,33 @@
         <v>14.19</v>
       </c>
       <c r="J23" t="n">
-        <v>12.61</v>
+        <v>12.69</v>
       </c>
       <c r="K23" t="n">
-        <v>12.5</v>
+        <v>11.8</v>
       </c>
       <c r="L23" t="n">
         <v>69.12</v>
       </c>
       <c r="M23" t="n">
-        <v>1.82</v>
+        <v>1.92</v>
       </c>
       <c r="N23" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>10-09-2026</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>0.455</v>
+        <v>0.49</v>
       </c>
       <c r="Q23" t="n">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="R23" t="n">
-        <v>1292</v>
+        <v>1265</v>
       </c>
       <c r="S23" t="n">
         <v>-61</v>
@@ -4663,10 +4663,10 @@
         <v>2.4</v>
       </c>
       <c r="AD23" t="n">
-        <v>12.57234083155615</v>
+        <v>12.64449812963585</v>
       </c>
       <c r="AE23" t="n">
-        <v>12.9</v>
+        <v>12.2</v>
       </c>
       <c r="AF23" t="inlineStr">
         <is>
@@ -4690,53 +4690,53 @@
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>10-09-2026</t>
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="AL23" t="n">
         <v>32</v>
       </c>
       <c r="AM23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AN23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AO23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AP23" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="AQ23" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="AR23" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="AS23" t="n">
-        <v>1817264</v>
+        <v>2767898</v>
       </c>
       <c r="AT23" t="n">
-        <v>4668828</v>
+        <v>5619462</v>
       </c>
       <c r="AU23" t="n">
-        <v>11285962</v>
+        <v>12236596</v>
       </c>
       <c r="AV23" t="n">
-        <v>18776351</v>
+        <v>19726985</v>
       </c>
       <c r="AW23" t="n">
-        <v>18776351</v>
+        <v>19726985</v>
       </c>
       <c r="AX23" t="n">
-        <v>1817264</v>
+        <v>2767898</v>
       </c>
       <c r="AY23" t="n">
-        <v>11285962</v>
+        <v>12236596</v>
       </c>
       <c r="AZ23" t="n">
         <v>1</v>
@@ -4745,7 +4745,7 @@
         <v>0</v>
       </c>
       <c r="BB23" t="n">
-        <v>0.161</v>
+        <v>0.2262</v>
       </c>
     </row>
     <row r="24">
@@ -4803,13 +4803,13 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>0.165</v>
+        <v>0.167</v>
       </c>
       <c r="Q24" t="n">
-        <v>672</v>
+        <v>664</v>
       </c>
       <c r="R24" t="n">
-        <v>56.1</v>
+        <v>55.5</v>
       </c>
       <c r="S24" t="n">
         <v>3</v>
@@ -4985,13 +4985,13 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>0.056</v>
+        <v>0.055</v>
       </c>
       <c r="Q25" t="n">
-        <v>1928</v>
+        <v>1976</v>
       </c>
       <c r="R25" t="n">
-        <v>44.2</v>
+        <v>45.4</v>
       </c>
       <c r="S25" t="n">
         <v>20</v>
@@ -5167,13 +5167,13 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>0.173</v>
+        <v>0.174</v>
       </c>
       <c r="Q26" t="n">
-        <v>888</v>
+        <v>884</v>
       </c>
       <c r="R26" t="n">
-        <v>8.73</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="S26" t="n">
         <v>7</v>
@@ -5349,13 +5349,13 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>0.438</v>
+        <v>0.446</v>
       </c>
       <c r="Q27" t="n">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="R27" t="n">
-        <v>38.8</v>
+        <v>38</v>
       </c>
       <c r="S27" t="n">
         <v>21</v>
@@ -5531,13 +5531,13 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>0.455</v>
+        <v>0.449</v>
       </c>
       <c r="Q28" t="n">
-        <v>1089</v>
+        <v>1102</v>
       </c>
       <c r="R28" t="n">
-        <v>55.5</v>
+        <v>56.1</v>
       </c>
       <c r="S28" t="n">
         <v>21</v>
@@ -5716,10 +5716,10 @@
         <v>0.045</v>
       </c>
       <c r="Q29" t="n">
-        <v>931</v>
+        <v>925</v>
       </c>
       <c r="R29" t="n">
-        <v>99.5</v>
+        <v>98.8</v>
       </c>
       <c r="S29" t="n">
         <v>15</v>
@@ -5898,7 +5898,7 @@
         <v>0.096</v>
       </c>
       <c r="Q30" t="n">
-        <v>1542</v>
+        <v>1535</v>
       </c>
       <c r="R30" t="n">
         <v>13.9</v>
@@ -6077,13 +6077,13 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>0.389</v>
+        <v>0.4</v>
       </c>
       <c r="Q31" t="n">
-        <v>422</v>
+        <v>410</v>
       </c>
       <c r="R31" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="S31" t="n">
         <v>246</v>
@@ -6259,13 +6259,13 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>0.265</v>
+        <v>0.263</v>
       </c>
       <c r="Q32" t="n">
-        <v>1122</v>
+        <v>1129</v>
       </c>
       <c r="R32" t="n">
-        <v>19.9</v>
+        <v>20.1</v>
       </c>
       <c r="S32" t="n">
         <v>12</v>
@@ -6444,10 +6444,10 @@
         <v>0.051</v>
       </c>
       <c r="Q33" t="n">
-        <v>5194</v>
+        <v>5120</v>
       </c>
       <c r="R33" t="n">
-        <v>33.8</v>
+        <v>33.4</v>
       </c>
       <c r="S33" t="n">
         <v>-25</v>
@@ -6626,7 +6626,7 @@
         <v>0.504</v>
       </c>
       <c r="Q34" t="n">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="R34" t="n">
         <v>14.9</v>
@@ -6805,13 +6805,13 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>0.95</v>
+        <v>0.964</v>
       </c>
       <c r="Q35" t="n">
-        <v>5097</v>
+        <v>5021</v>
       </c>
       <c r="R35" t="n">
-        <v>40.9</v>
+        <v>40.3</v>
       </c>
       <c r="S35" t="n">
         <v>0</v>
@@ -6987,10 +6987,10 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>1.559</v>
+        <v>1.573</v>
       </c>
       <c r="Q36" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="n">
@@ -7167,13 +7167,13 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>0.034</v>
+        <v>0.035</v>
       </c>
       <c r="Q37" t="n">
-        <v>3166</v>
+        <v>3103</v>
       </c>
       <c r="R37" t="n">
-        <v>21.4</v>
+        <v>21</v>
       </c>
       <c r="S37" t="n">
         <v>17</v>
@@ -7352,10 +7352,10 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="Q38" t="n">
-        <v>54079</v>
+        <v>53951</v>
       </c>
       <c r="R38" t="n">
-        <v>45.8</v>
+        <v>45.7</v>
       </c>
       <c r="S38" t="n">
         <v>5</v>
@@ -7531,13 +7531,13 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>0.183</v>
+        <v>0.186</v>
       </c>
       <c r="Q39" t="n">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="R39" t="n">
-        <v>24.4</v>
+        <v>24.1</v>
       </c>
       <c r="S39" t="n">
         <v>12</v>
@@ -7713,13 +7713,13 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>0.452</v>
+        <v>0.456</v>
       </c>
       <c r="Q40" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="R40" t="n">
-        <v>74.90000000000001</v>
+        <v>74.2</v>
       </c>
       <c r="S40" t="n">
         <v>-1</v>
@@ -7898,10 +7898,10 @@
         <v>0.002</v>
       </c>
       <c r="Q41" t="n">
-        <v>327539</v>
+        <v>329045</v>
       </c>
       <c r="R41" t="n">
-        <v>18</v>
+        <v>18.1</v>
       </c>
       <c r="S41" t="n">
         <v>7</v>
@@ -8077,13 +8077,13 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>0.159</v>
+        <v>0.16</v>
       </c>
       <c r="Q42" t="n">
-        <v>779</v>
+        <v>775</v>
       </c>
       <c r="R42" t="n">
-        <v>14.2</v>
+        <v>14.1</v>
       </c>
       <c r="S42" t="n">
         <v>185</v>
@@ -8260,10 +8260,10 @@
         <v>0.037</v>
       </c>
       <c r="Q43" t="n">
-        <v>838</v>
+        <v>827</v>
       </c>
       <c r="R43" t="n">
-        <v>20.1</v>
+        <v>19.8</v>
       </c>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="n">
@@ -8431,13 +8431,13 @@
         </is>
       </c>
       <c r="P44" t="n">
-        <v>0.284</v>
+        <v>0.285</v>
       </c>
       <c r="Q44" t="n">
-        <v>3599</v>
+        <v>3583</v>
       </c>
       <c r="R44" t="n">
-        <v>25.2</v>
+        <v>25</v>
       </c>
       <c r="S44" t="n">
         <v>2</v>
@@ -8613,13 +8613,13 @@
         </is>
       </c>
       <c r="P45" t="n">
-        <v>0.128</v>
+        <v>0.13</v>
       </c>
       <c r="Q45" t="n">
-        <v>576</v>
+        <v>570</v>
       </c>
       <c r="R45" t="n">
-        <v>13.6</v>
+        <v>13.5</v>
       </c>
       <c r="S45" t="n">
         <v>61</v>
@@ -8793,13 +8793,13 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>0.19</v>
+        <v>0.192</v>
       </c>
       <c r="Q46" t="n">
-        <v>473</v>
+        <v>468</v>
       </c>
       <c r="R46" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="S46" t="n">
         <v>19</v>
@@ -8975,13 +8975,13 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>0.6</v>
+        <v>0.614</v>
       </c>
       <c r="Q47" t="n">
-        <v>1813</v>
+        <v>1771</v>
       </c>
       <c r="R47" t="n">
-        <v>32.7</v>
+        <v>31.9</v>
       </c>
       <c r="S47" t="n">
         <v>39</v>
@@ -9157,13 +9157,13 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="Q48" t="n">
-        <v>1482</v>
+        <v>1464</v>
       </c>
       <c r="R48" t="n">
-        <v>18.8</v>
+        <v>18.6</v>
       </c>
       <c r="S48" t="n">
         <v>13</v>
@@ -9339,13 +9339,13 @@
         </is>
       </c>
       <c r="P49" t="n">
-        <v>0.266</v>
+        <v>0.268</v>
       </c>
       <c r="Q49" t="n">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="R49" t="n">
-        <v>15.5</v>
+        <v>15.3</v>
       </c>
       <c r="S49" t="n">
         <v>16</v>
@@ -9521,13 +9521,13 @@
         </is>
       </c>
       <c r="P50" t="n">
-        <v>0.055</v>
+        <v>0.053</v>
       </c>
       <c r="Q50" t="n">
-        <v>861</v>
+        <v>890</v>
       </c>
       <c r="R50" t="n">
-        <v>23.4</v>
+        <v>24.3</v>
       </c>
       <c r="S50" t="n">
         <v>9</v>
@@ -10393,7 +10393,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PNGS Reva Diamond Jewellery Limited</t>
+          <t>PNGS REVA DIAMOND JEWELLERY LIMITED</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -10470,23 +10470,23 @@
         <v>14.19</v>
       </c>
       <c r="D23" t="n">
-        <v>12.61</v>
+        <v>12.69</v>
       </c>
       <c r="E23" t="n">
-        <v>12.5</v>
+        <v>11.8</v>
       </c>
       <c r="F23" t="n">
         <v>69.12</v>
       </c>
       <c r="G23" t="n">
-        <v>1.82</v>
+        <v>1.92</v>
       </c>
       <c r="H23" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>10-09-2026</t>
         </is>
       </c>
     </row>

</xml_diff>